<commit_message>
Add PiN step 1 hybrid for South_Sudan___SSD
</commit_message>
<xml_diff>
--- a/platform_PiN_output/South_Sudan___SSD/PiN_step1_South_Sudan___SSD_1028_03PM.xlsx
+++ b/platform_PiN_output/South_Sudan___SSD/PiN_step1_South_Sudan___SSD_1028_03PM.xlsx
@@ -1479,38 +1479,38 @@
         <v>173762</v>
       </c>
       <c r="D4" s="33" t="n">
-        <v>48.2</v>
+        <v>64.5</v>
       </c>
       <c r="E4" s="33" t="n">
-        <v>83744</v>
+        <v>112054</v>
       </c>
       <c r="F4" s="33" t="n">
-        <v>33.6</v>
+        <v>10.5</v>
       </c>
       <c r="G4" s="33" t="n">
-        <v>58408</v>
+        <v>18216</v>
       </c>
       <c r="H4" s="33" t="n">
-        <v>2</v>
+        <v>2.5</v>
       </c>
       <c r="I4" s="33" t="n">
-        <v>3431</v>
+        <v>4325</v>
       </c>
       <c r="J4" s="33" t="n">
-        <v>16.2</v>
+        <v>22.5</v>
       </c>
       <c r="K4" s="33" t="n">
-        <v>28180</v>
+        <v>39167</v>
       </c>
       <c r="L4" s="33" t="n">
-        <v>51.8</v>
+        <v>35.5</v>
       </c>
       <c r="M4" s="33" t="n">
-        <v>90019</v>
+        <v>61708</v>
       </c>
       <c r="N4" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O4" s="35" t="n">
@@ -1774,34 +1774,34 @@
         <v>22759</v>
       </c>
       <c r="D5" s="33" t="n">
-        <v>48.2</v>
+        <v>35.4</v>
       </c>
       <c r="E5" s="33" t="n">
-        <v>10969</v>
+        <v>8059</v>
       </c>
       <c r="F5" s="33" t="n">
-        <v>33.6</v>
+        <v>49.2</v>
       </c>
       <c r="G5" s="33" t="n">
-        <v>7650</v>
+        <v>11207</v>
       </c>
       <c r="H5" s="33" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="I5" s="33" t="n">
-        <v>449</v>
+        <v>0</v>
       </c>
       <c r="J5" s="33" t="n">
-        <v>16.2</v>
+        <v>15.4</v>
       </c>
       <c r="K5" s="33" t="n">
-        <v>3691</v>
+        <v>3494</v>
       </c>
       <c r="L5" s="33" t="n">
-        <v>51.8</v>
+        <v>64.59999999999999</v>
       </c>
       <c r="M5" s="33" t="n">
-        <v>11791</v>
+        <v>14700</v>
       </c>
       <c r="N5" s="34" t="inlineStr">
         <is>
@@ -2033,34 +2033,34 @@
         <v>20528</v>
       </c>
       <c r="D6" s="33" t="n">
-        <v>48.2</v>
+        <v>38.3</v>
       </c>
       <c r="E6" s="33" t="n">
-        <v>9893</v>
+        <v>7862</v>
       </c>
       <c r="F6" s="33" t="n">
-        <v>33.6</v>
+        <v>51.5</v>
       </c>
       <c r="G6" s="33" t="n">
-        <v>6900</v>
+        <v>10565</v>
       </c>
       <c r="H6" s="33" t="n">
-        <v>2</v>
+        <v>5.9</v>
       </c>
       <c r="I6" s="33" t="n">
-        <v>405</v>
+        <v>1215</v>
       </c>
       <c r="J6" s="33" t="n">
-        <v>16.2</v>
+        <v>4.3</v>
       </c>
       <c r="K6" s="33" t="n">
-        <v>3329</v>
+        <v>886</v>
       </c>
       <c r="L6" s="33" t="n">
-        <v>51.8</v>
+        <v>61.7</v>
       </c>
       <c r="M6" s="33" t="n">
-        <v>10635</v>
+        <v>12666</v>
       </c>
       <c r="N6" s="34" t="inlineStr">
         <is>
@@ -2310,34 +2310,34 @@
         <v>34047</v>
       </c>
       <c r="D7" s="33" t="n">
-        <v>48.2</v>
+        <v>48.1</v>
       </c>
       <c r="E7" s="33" t="n">
-        <v>16409</v>
+        <v>16360</v>
       </c>
       <c r="F7" s="33" t="n">
-        <v>33.6</v>
+        <v>49.6</v>
       </c>
       <c r="G7" s="33" t="n">
-        <v>11444</v>
+        <v>16899</v>
       </c>
       <c r="H7" s="33" t="n">
-        <v>2</v>
+        <v>2.3</v>
       </c>
       <c r="I7" s="33" t="n">
-        <v>672</v>
+        <v>788</v>
       </c>
       <c r="J7" s="33" t="n">
-        <v>16.2</v>
+        <v>0</v>
       </c>
       <c r="K7" s="33" t="n">
-        <v>5522</v>
+        <v>0</v>
       </c>
       <c r="L7" s="33" t="n">
-        <v>51.8</v>
+        <v>51.9</v>
       </c>
       <c r="M7" s="33" t="n">
-        <v>17638</v>
+        <v>17687</v>
       </c>
       <c r="N7" s="34" t="inlineStr">
         <is>
@@ -2569,34 +2569,34 @@
         <v>73580</v>
       </c>
       <c r="D8" s="33" t="n">
-        <v>48.2</v>
+        <v>23.1</v>
       </c>
       <c r="E8" s="33" t="n">
-        <v>35461</v>
+        <v>16991</v>
       </c>
       <c r="F8" s="33" t="n">
-        <v>33.6</v>
+        <v>64.7</v>
       </c>
       <c r="G8" s="33" t="n">
-        <v>24733</v>
+        <v>47629</v>
       </c>
       <c r="H8" s="33" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="I8" s="33" t="n">
-        <v>1453</v>
+        <v>1091</v>
       </c>
       <c r="J8" s="33" t="n">
-        <v>16.2</v>
+        <v>10.7</v>
       </c>
       <c r="K8" s="33" t="n">
-        <v>11933</v>
+        <v>7869</v>
       </c>
       <c r="L8" s="33" t="n">
-        <v>51.8</v>
+        <v>76.90000000000001</v>
       </c>
       <c r="M8" s="33" t="n">
-        <v>38119</v>
+        <v>56589</v>
       </c>
       <c r="N8" s="34" t="inlineStr">
         <is>
@@ -2850,38 +2850,38 @@
         <v>87932</v>
       </c>
       <c r="D9" s="33" t="n">
-        <v>48.2</v>
+        <v>47.7</v>
       </c>
       <c r="E9" s="33" t="n">
-        <v>42378</v>
+        <v>41902</v>
       </c>
       <c r="F9" s="33" t="n">
-        <v>33.6</v>
+        <v>31.3</v>
       </c>
       <c r="G9" s="33" t="n">
-        <v>29557</v>
+        <v>27536</v>
       </c>
       <c r="H9" s="33" t="n">
         <v>2</v>
       </c>
       <c r="I9" s="33" t="n">
-        <v>1736</v>
+        <v>1767</v>
       </c>
       <c r="J9" s="33" t="n">
-        <v>16.2</v>
+        <v>19</v>
       </c>
       <c r="K9" s="33" t="n">
-        <v>14261</v>
+        <v>16728</v>
       </c>
       <c r="L9" s="33" t="n">
-        <v>51.8</v>
+        <v>52.3</v>
       </c>
       <c r="M9" s="33" t="n">
-        <v>45554</v>
+        <v>46030</v>
       </c>
       <c r="N9" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O9" s="35" t="n">
@@ -3141,34 +3141,34 @@
         <v>31738</v>
       </c>
       <c r="D10" s="33" t="n">
-        <v>31.5</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="E10" s="33" t="n">
-        <v>9995</v>
+        <v>3063</v>
       </c>
       <c r="F10" s="33" t="n">
-        <v>62.3</v>
+        <v>90.3</v>
       </c>
       <c r="G10" s="33" t="n">
-        <v>19774</v>
+        <v>28675</v>
       </c>
       <c r="H10" s="33" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="I10" s="33" t="n">
-        <v>1109</v>
+        <v>0</v>
       </c>
       <c r="J10" s="33" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="K10" s="33" t="n">
-        <v>859</v>
+        <v>0</v>
       </c>
       <c r="L10" s="33" t="n">
-        <v>68.5</v>
+        <v>90.3</v>
       </c>
       <c r="M10" s="33" t="n">
-        <v>21743</v>
+        <v>28675</v>
       </c>
       <c r="N10" s="34" t="inlineStr">
         <is>
@@ -3415,42 +3415,40 @@
         </is>
       </c>
       <c r="C11" s="33" t="n">
-        <v>27970</v>
+        <v/>
       </c>
       <c r="D11" s="33" t="n">
-        <v>31.5</v>
+        <v/>
       </c>
       <c r="E11" s="33" t="n">
-        <v>8809</v>
+        <v/>
       </c>
       <c r="F11" s="33" t="n">
-        <v>62.3</v>
+        <v/>
       </c>
       <c r="G11" s="33" t="n">
-        <v>17427</v>
+        <v/>
       </c>
       <c r="H11" s="33" t="n">
-        <v>3.5</v>
+        <v/>
       </c>
       <c r="I11" s="33" t="n">
-        <v>978</v>
+        <v/>
       </c>
       <c r="J11" s="33" t="n">
-        <v>2.7</v>
+        <v/>
       </c>
       <c r="K11" s="33" t="n">
-        <v>757</v>
+        <v/>
       </c>
       <c r="L11" s="33" t="n">
-        <v>68.5</v>
+        <v/>
       </c>
       <c r="M11" s="33" t="n">
-        <v>19162</v>
-      </c>
-      <c r="N11" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N11" s="34" t="n">
+        <v/>
       </c>
       <c r="O11" s="35" t="n">
         <v/>
@@ -3658,8 +3656,10 @@
       <c r="CB11" s="48" t="n">
         <v>0.07307042667254167</v>
       </c>
-      <c r="CC11" s="49" t="n">
-        <v>0.069442286204721</v>
+      <c r="CC11" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="12">
@@ -3677,34 +3677,34 @@
         <v>48380</v>
       </c>
       <c r="D12" s="33" t="n">
-        <v>31.5</v>
+        <v>0</v>
       </c>
       <c r="E12" s="33" t="n">
-        <v>15236</v>
+        <v>0</v>
       </c>
       <c r="F12" s="33" t="n">
-        <v>62.3</v>
+        <v>85.40000000000001</v>
       </c>
       <c r="G12" s="33" t="n">
-        <v>30143</v>
+        <v>41313</v>
       </c>
       <c r="H12" s="33" t="n">
-        <v>3.5</v>
+        <v>4.6</v>
       </c>
       <c r="I12" s="33" t="n">
-        <v>1691</v>
+        <v>2221</v>
       </c>
       <c r="J12" s="33" t="n">
-        <v>2.7</v>
+        <v>10</v>
       </c>
       <c r="K12" s="33" t="n">
-        <v>1310</v>
+        <v>4846</v>
       </c>
       <c r="L12" s="33" t="n">
-        <v>68.5</v>
+        <v>100</v>
       </c>
       <c r="M12" s="33" t="n">
-        <v>33144</v>
+        <v>48380</v>
       </c>
       <c r="N12" s="34" t="inlineStr">
         <is>
@@ -3958,34 +3958,34 @@
         <v>49084</v>
       </c>
       <c r="D13" s="33" t="n">
-        <v>31.5</v>
+        <v>0</v>
       </c>
       <c r="E13" s="33" t="n">
-        <v>15458</v>
+        <v>0</v>
       </c>
       <c r="F13" s="33" t="n">
-        <v>62.3</v>
+        <v>100</v>
       </c>
       <c r="G13" s="33" t="n">
-        <v>30582</v>
+        <v>49084</v>
       </c>
       <c r="H13" s="33" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="I13" s="33" t="n">
-        <v>1716</v>
+        <v>0</v>
       </c>
       <c r="J13" s="33" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="K13" s="33" t="n">
-        <v>1329</v>
+        <v>0</v>
       </c>
       <c r="L13" s="33" t="n">
-        <v>68.5</v>
+        <v>100</v>
       </c>
       <c r="M13" s="33" t="n">
-        <v>33627</v>
+        <v>49084</v>
       </c>
       <c r="N13" s="34" t="inlineStr">
         <is>
@@ -4217,34 +4217,34 @@
         <v>39536</v>
       </c>
       <c r="D14" s="33" t="n">
-        <v>31.5</v>
+        <v>41.4</v>
       </c>
       <c r="E14" s="33" t="n">
-        <v>12451</v>
+        <v>16377</v>
       </c>
       <c r="F14" s="33" t="n">
-        <v>62.3</v>
+        <v>58.6</v>
       </c>
       <c r="G14" s="33" t="n">
-        <v>24633</v>
+        <v>23160</v>
       </c>
       <c r="H14" s="33" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="I14" s="33" t="n">
-        <v>1382</v>
+        <v>0</v>
       </c>
       <c r="J14" s="33" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="K14" s="33" t="n">
-        <v>1071</v>
+        <v>0</v>
       </c>
       <c r="L14" s="33" t="n">
-        <v>68.5</v>
+        <v>58.6</v>
       </c>
       <c r="M14" s="33" t="n">
-        <v>27086</v>
+        <v>23160</v>
       </c>
       <c r="N14" s="34" t="inlineStr">
         <is>
@@ -4476,38 +4476,38 @@
         <v>44227</v>
       </c>
       <c r="D15" s="33" t="n">
-        <v>31.5</v>
+        <v>83.8</v>
       </c>
       <c r="E15" s="33" t="n">
-        <v>13928</v>
+        <v>37056</v>
       </c>
       <c r="F15" s="33" t="n">
-        <v>62.3</v>
+        <v>16.2</v>
       </c>
       <c r="G15" s="33" t="n">
-        <v>27555</v>
+        <v>7171</v>
       </c>
       <c r="H15" s="33" t="n">
-        <v>3.5</v>
+        <v>0</v>
       </c>
       <c r="I15" s="33" t="n">
-        <v>1546</v>
+        <v>0</v>
       </c>
       <c r="J15" s="33" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="K15" s="33" t="n">
-        <v>1198</v>
+        <v>0</v>
       </c>
       <c r="L15" s="33" t="n">
-        <v>68.5</v>
+        <v>16.2</v>
       </c>
       <c r="M15" s="33" t="n">
-        <v>30299</v>
+        <v>7171</v>
       </c>
       <c r="N15" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="O15" s="35" t="n">
@@ -4735,34 +4735,34 @@
         <v>72762</v>
       </c>
       <c r="D16" s="33" t="n">
-        <v>31.5</v>
+        <v>78.90000000000001</v>
       </c>
       <c r="E16" s="33" t="n">
-        <v>22915</v>
+        <v>57412</v>
       </c>
       <c r="F16" s="33" t="n">
-        <v>62.3</v>
+        <v>5.2</v>
       </c>
       <c r="G16" s="33" t="n">
-        <v>45334</v>
+        <v>3784</v>
       </c>
       <c r="H16" s="33" t="n">
-        <v>3.5</v>
+        <v>15.9</v>
       </c>
       <c r="I16" s="33" t="n">
-        <v>2543</v>
+        <v>11566</v>
       </c>
       <c r="J16" s="33" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="K16" s="33" t="n">
-        <v>1970</v>
+        <v>0</v>
       </c>
       <c r="L16" s="33" t="n">
-        <v>68.5</v>
+        <v>21.1</v>
       </c>
       <c r="M16" s="33" t="n">
-        <v>49848</v>
+        <v>15350</v>
       </c>
       <c r="N16" s="34" t="inlineStr">
         <is>
@@ -4994,34 +4994,34 @@
         <v>19590</v>
       </c>
       <c r="D17" s="33" t="n">
-        <v>31.5</v>
+        <v>66.2</v>
       </c>
       <c r="E17" s="33" t="n">
-        <v>6169</v>
+        <v>12965</v>
       </c>
       <c r="F17" s="33" t="n">
-        <v>62.3</v>
+        <v>30.8</v>
       </c>
       <c r="G17" s="33" t="n">
-        <v>12206</v>
+        <v>6038</v>
       </c>
       <c r="H17" s="33" t="n">
-        <v>3.5</v>
+        <v>3</v>
       </c>
       <c r="I17" s="33" t="n">
-        <v>685</v>
+        <v>587</v>
       </c>
       <c r="J17" s="33" t="n">
-        <v>2.7</v>
+        <v>0</v>
       </c>
       <c r="K17" s="33" t="n">
-        <v>531</v>
+        <v>0</v>
       </c>
       <c r="L17" s="33" t="n">
-        <v>68.5</v>
+        <v>33.8</v>
       </c>
       <c r="M17" s="33" t="n">
-        <v>13421</v>
+        <v>6625</v>
       </c>
       <c r="N17" s="34" t="inlineStr">
         <is>
@@ -5253,34 +5253,34 @@
         <v>66998</v>
       </c>
       <c r="D18" s="33" t="n">
-        <v>35.2</v>
+        <v>41.3</v>
       </c>
       <c r="E18" s="33" t="n">
-        <v>23568</v>
+        <v>27645</v>
       </c>
       <c r="F18" s="33" t="n">
-        <v>54.3</v>
+        <v>44</v>
       </c>
       <c r="G18" s="33" t="n">
-        <v>36406</v>
+        <v>29492</v>
       </c>
       <c r="H18" s="33" t="n">
-        <v>7.2</v>
+        <v>13.1</v>
       </c>
       <c r="I18" s="33" t="n">
-        <v>4825</v>
+        <v>8788</v>
       </c>
       <c r="J18" s="33" t="n">
-        <v>3.3</v>
+        <v>1.6</v>
       </c>
       <c r="K18" s="33" t="n">
-        <v>2199</v>
+        <v>1073</v>
       </c>
       <c r="L18" s="33" t="n">
-        <v>64.8</v>
+        <v>58.7</v>
       </c>
       <c r="M18" s="33" t="n">
-        <v>43430</v>
+        <v>39354</v>
       </c>
       <c r="N18" s="34" t="inlineStr">
         <is>
@@ -5532,34 +5532,34 @@
         <v>53607</v>
       </c>
       <c r="D19" s="33" t="n">
-        <v>35.2</v>
+        <v>56.9</v>
       </c>
       <c r="E19" s="33" t="n">
-        <v>18858</v>
+        <v>30477</v>
       </c>
       <c r="F19" s="33" t="n">
-        <v>54.3</v>
+        <v>36.2</v>
       </c>
       <c r="G19" s="33" t="n">
-        <v>29129</v>
+        <v>19385</v>
       </c>
       <c r="H19" s="33" t="n">
-        <v>7.2</v>
+        <v>2.6</v>
       </c>
       <c r="I19" s="33" t="n">
-        <v>3861</v>
+        <v>1395</v>
       </c>
       <c r="J19" s="33" t="n">
-        <v>3.3</v>
+        <v>4.4</v>
       </c>
       <c r="K19" s="33" t="n">
-        <v>1759</v>
+        <v>2349</v>
       </c>
       <c r="L19" s="33" t="n">
-        <v>64.8</v>
+        <v>43.1</v>
       </c>
       <c r="M19" s="33" t="n">
-        <v>34749</v>
+        <v>23130</v>
       </c>
       <c r="N19" s="34" t="inlineStr">
         <is>
@@ -5791,34 +5791,34 @@
         <v>97707</v>
       </c>
       <c r="D20" s="33" t="n">
-        <v>35.2</v>
+        <v>37</v>
       </c>
       <c r="E20" s="33" t="n">
-        <v>34371</v>
+        <v>36115</v>
       </c>
       <c r="F20" s="33" t="n">
-        <v>54.3</v>
+        <v>54.9</v>
       </c>
       <c r="G20" s="33" t="n">
-        <v>53092</v>
+        <v>53605</v>
       </c>
       <c r="H20" s="33" t="n">
-        <v>7.2</v>
+        <v>4.5</v>
       </c>
       <c r="I20" s="33" t="n">
-        <v>7037</v>
+        <v>4435</v>
       </c>
       <c r="J20" s="33" t="n">
-        <v>3.3</v>
+        <v>3.6</v>
       </c>
       <c r="K20" s="33" t="n">
-        <v>3206</v>
+        <v>3551</v>
       </c>
       <c r="L20" s="33" t="n">
-        <v>64.8</v>
+        <v>63</v>
       </c>
       <c r="M20" s="33" t="n">
-        <v>63336</v>
+        <v>61591</v>
       </c>
       <c r="N20" s="34" t="inlineStr">
         <is>
@@ -6065,41 +6065,61 @@
         </is>
       </c>
       <c r="C21" s="33" t="n">
-        <v>30387</v>
-      </c>
-      <c r="D21" s="33" t="n">
-        <v>35.2</v>
-      </c>
-      <c r="E21" s="33" t="n">
-        <v>10690</v>
-      </c>
-      <c r="F21" s="33" t="n">
-        <v>54.3</v>
-      </c>
-      <c r="G21" s="33" t="n">
-        <v>16512</v>
-      </c>
-      <c r="H21" s="33" t="n">
-        <v>7.2</v>
-      </c>
-      <c r="I21" s="33" t="n">
-        <v>2189</v>
-      </c>
-      <c r="J21" s="33" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="K21" s="33" t="n">
-        <v>997</v>
-      </c>
-      <c r="L21" s="33" t="n">
-        <v>64.8</v>
-      </c>
-      <c r="M21" s="33" t="n">
-        <v>19698</v>
+        <v/>
+      </c>
+      <c r="D21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="E21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="F21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="G21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="H21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="I21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="J21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="K21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="L21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="M21" s="33" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
       </c>
       <c r="N21" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>Missing MSNA data for 2024 AND 2025</t>
         </is>
       </c>
       <c r="O21" s="35" t="n">
@@ -6124,53 +6144,85 @@
         <v/>
       </c>
       <c r="V21" s="39" t="inlineStr"/>
-      <c r="W21" s="40" t="n">
-        <v/>
-      </c>
-      <c r="X21" s="40" t="n">
-        <v/>
-      </c>
-      <c r="Y21" s="40" t="n">
-        <v/>
-      </c>
-      <c r="Z21" s="40" t="n">
-        <v/>
-      </c>
-      <c r="AA21" s="41" t="n">
-        <v/>
-      </c>
-      <c r="AB21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AC21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AD21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AE21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AF21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AG21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AH21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AI21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AJ21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AK21" s="42" t="n">
-        <v/>
-      </c>
-      <c r="AL21" s="43" t="n">
-        <v/>
+      <c r="W21" s="40" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="X21" s="40" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="Y21" s="40" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="Z21" s="40" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AA21" s="41" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AB21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AC21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AD21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AE21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AF21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AG21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AH21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AI21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AJ21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AK21" s="42" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
+      </c>
+      <c r="AL21" s="43" t="inlineStr">
+        <is>
+          <t>Missing MSNA data for 2024 AND 2025</t>
+        </is>
       </c>
       <c r="AM21" s="44" t="n">
         <v/>
@@ -6298,8 +6350,10 @@
       <c r="CB21" s="48" t="n">
         <v/>
       </c>
-      <c r="CC21" s="49" t="n">
-        <v>0.6702445521486068</v>
+      <c r="CC21" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="22">
@@ -6314,42 +6368,40 @@
         </is>
       </c>
       <c r="C22" s="33" t="n">
-        <v>61048</v>
+        <v/>
       </c>
       <c r="D22" s="33" t="n">
-        <v>35.2</v>
+        <v/>
       </c>
       <c r="E22" s="33" t="n">
-        <v>21475</v>
+        <v/>
       </c>
       <c r="F22" s="33" t="n">
-        <v>54.3</v>
+        <v/>
       </c>
       <c r="G22" s="33" t="n">
-        <v>33172</v>
+        <v/>
       </c>
       <c r="H22" s="33" t="n">
-        <v>7.2</v>
+        <v/>
       </c>
       <c r="I22" s="33" t="n">
-        <v>4397</v>
+        <v/>
       </c>
       <c r="J22" s="33" t="n">
-        <v>3.3</v>
+        <v/>
       </c>
       <c r="K22" s="33" t="n">
-        <v>2003</v>
+        <v/>
       </c>
       <c r="L22" s="33" t="n">
-        <v>64.8</v>
+        <v/>
       </c>
       <c r="M22" s="33" t="n">
-        <v>39573</v>
-      </c>
-      <c r="N22" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N22" s="34" t="n">
+        <v/>
       </c>
       <c r="O22" s="35" t="n">
         <v/>
@@ -6557,8 +6609,10 @@
       <c r="CB22" s="48" t="n">
         <v>0.3386086896360869</v>
       </c>
-      <c r="CC22" s="49" t="n">
-        <v>0.4229119464449064</v>
+      <c r="CC22" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="23">
@@ -6573,42 +6627,40 @@
         </is>
       </c>
       <c r="C23" s="33" t="n">
-        <v>78443</v>
+        <v/>
       </c>
       <c r="D23" s="33" t="n">
-        <v>35.2</v>
+        <v/>
       </c>
       <c r="E23" s="33" t="n">
-        <v>27594</v>
+        <v/>
       </c>
       <c r="F23" s="33" t="n">
-        <v>54.3</v>
+        <v/>
       </c>
       <c r="G23" s="33" t="n">
-        <v>42625</v>
+        <v/>
       </c>
       <c r="H23" s="33" t="n">
-        <v>7.2</v>
+        <v/>
       </c>
       <c r="I23" s="33" t="n">
-        <v>5650</v>
+        <v/>
       </c>
       <c r="J23" s="33" t="n">
-        <v>3.3</v>
+        <v/>
       </c>
       <c r="K23" s="33" t="n">
-        <v>2574</v>
+        <v/>
       </c>
       <c r="L23" s="33" t="n">
-        <v>64.8</v>
+        <v/>
       </c>
       <c r="M23" s="33" t="n">
-        <v>50849</v>
-      </c>
-      <c r="N23" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N23" s="34" t="n">
+        <v/>
       </c>
       <c r="O23" s="35" t="n">
         <v/>
@@ -6836,8 +6888,10 @@
       <c r="CB23" s="48" t="n">
         <v>0.4775064356780074</v>
       </c>
-      <c r="CC23" s="49" t="n">
-        <v>0.5661324713912752</v>
+      <c r="CC23" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="24">
@@ -6855,34 +6909,34 @@
         <v>53757</v>
       </c>
       <c r="D24" s="33" t="n">
-        <v>35.2</v>
+        <v>15.1</v>
       </c>
       <c r="E24" s="33" t="n">
-        <v>18910</v>
+        <v>8138</v>
       </c>
       <c r="F24" s="33" t="n">
-        <v>54.3</v>
+        <v>69.7</v>
       </c>
       <c r="G24" s="33" t="n">
-        <v>29211</v>
+        <v>37462</v>
       </c>
       <c r="H24" s="33" t="n">
-        <v>7.2</v>
+        <v>8.4</v>
       </c>
       <c r="I24" s="33" t="n">
-        <v>3872</v>
+        <v>4497</v>
       </c>
       <c r="J24" s="33" t="n">
-        <v>3.3</v>
+        <v>6.8</v>
       </c>
       <c r="K24" s="33" t="n">
-        <v>1764</v>
+        <v>3660</v>
       </c>
       <c r="L24" s="33" t="n">
-        <v>64.8</v>
+        <v>84.90000000000001</v>
       </c>
       <c r="M24" s="33" t="n">
-        <v>34846</v>
+        <v>45619</v>
       </c>
       <c r="N24" s="34" t="inlineStr">
         <is>
@@ -7134,34 +7188,34 @@
         <v>57769</v>
       </c>
       <c r="D25" s="33" t="n">
-        <v>35.2</v>
+        <v>2.2</v>
       </c>
       <c r="E25" s="33" t="n">
-        <v>20322</v>
+        <v>1298</v>
       </c>
       <c r="F25" s="33" t="n">
-        <v>54.3</v>
+        <v>95.09999999999999</v>
       </c>
       <c r="G25" s="33" t="n">
-        <v>31391</v>
+        <v>54917</v>
       </c>
       <c r="H25" s="33" t="n">
-        <v>7.2</v>
+        <v>2.7</v>
       </c>
       <c r="I25" s="33" t="n">
-        <v>4161</v>
+        <v>1555</v>
       </c>
       <c r="J25" s="33" t="n">
-        <v>3.3</v>
+        <v>0</v>
       </c>
       <c r="K25" s="33" t="n">
-        <v>1896</v>
+        <v>0</v>
       </c>
       <c r="L25" s="33" t="n">
-        <v>64.8</v>
+        <v>97.8</v>
       </c>
       <c r="M25" s="33" t="n">
-        <v>37447</v>
+        <v>56471</v>
       </c>
       <c r="N25" s="34" t="inlineStr">
         <is>
@@ -7411,34 +7465,34 @@
         <v>25482</v>
       </c>
       <c r="D26" s="33" t="n">
-        <v>35.2</v>
+        <v>65.3</v>
       </c>
       <c r="E26" s="33" t="n">
-        <v>8964</v>
+        <v>16633</v>
       </c>
       <c r="F26" s="33" t="n">
-        <v>54.3</v>
+        <v>31.3</v>
       </c>
       <c r="G26" s="33" t="n">
-        <v>13846</v>
+        <v>7969</v>
       </c>
       <c r="H26" s="33" t="n">
-        <v>7.2</v>
+        <v>3</v>
       </c>
       <c r="I26" s="33" t="n">
-        <v>1835</v>
+        <v>764</v>
       </c>
       <c r="J26" s="33" t="n">
-        <v>3.3</v>
+        <v>0.5</v>
       </c>
       <c r="K26" s="33" t="n">
-        <v>836</v>
+        <v>116</v>
       </c>
       <c r="L26" s="33" t="n">
-        <v>64.8</v>
+        <v>34.7</v>
       </c>
       <c r="M26" s="33" t="n">
-        <v>16518</v>
+        <v>8849</v>
       </c>
       <c r="N26" s="34" t="inlineStr">
         <is>
@@ -7687,42 +7741,40 @@
         </is>
       </c>
       <c r="C27" s="33" t="n">
-        <v>35288</v>
+        <v/>
       </c>
       <c r="D27" s="33" t="n">
-        <v>35.2</v>
+        <v/>
       </c>
       <c r="E27" s="33" t="n">
-        <v>12413</v>
+        <v/>
       </c>
       <c r="F27" s="33" t="n">
-        <v>54.3</v>
+        <v/>
       </c>
       <c r="G27" s="33" t="n">
-        <v>19175</v>
+        <v/>
       </c>
       <c r="H27" s="33" t="n">
-        <v>7.2</v>
+        <v/>
       </c>
       <c r="I27" s="33" t="n">
-        <v>2541</v>
+        <v/>
       </c>
       <c r="J27" s="33" t="n">
-        <v>3.3</v>
+        <v/>
       </c>
       <c r="K27" s="33" t="n">
-        <v>1158</v>
+        <v/>
       </c>
       <c r="L27" s="33" t="n">
-        <v>64.8</v>
+        <v/>
       </c>
       <c r="M27" s="33" t="n">
-        <v>22874</v>
-      </c>
-      <c r="N27" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N27" s="34" t="n">
+        <v/>
       </c>
       <c r="O27" s="35" t="n">
         <v/>
@@ -7930,8 +7982,10 @@
       <c r="CB27" s="48" t="n">
         <v>0.1717686573760349</v>
       </c>
-      <c r="CC27" s="49" t="n">
-        <v>0.2382611590554925</v>
+      <c r="CC27" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="28">
@@ -7946,42 +8000,40 @@
         </is>
       </c>
       <c r="C28" s="33" t="n">
-        <v>53509</v>
+        <v/>
       </c>
       <c r="D28" s="33" t="n">
-        <v>35.2</v>
+        <v/>
       </c>
       <c r="E28" s="33" t="n">
-        <v>18823</v>
+        <v/>
       </c>
       <c r="F28" s="33" t="n">
-        <v>54.3</v>
+        <v/>
       </c>
       <c r="G28" s="33" t="n">
-        <v>29076</v>
+        <v/>
       </c>
       <c r="H28" s="33" t="n">
-        <v>7.2</v>
+        <v/>
       </c>
       <c r="I28" s="33" t="n">
-        <v>3854</v>
+        <v/>
       </c>
       <c r="J28" s="33" t="n">
-        <v>3.3</v>
+        <v/>
       </c>
       <c r="K28" s="33" t="n">
-        <v>1756</v>
+        <v/>
       </c>
       <c r="L28" s="33" t="n">
-        <v>64.8</v>
+        <v/>
       </c>
       <c r="M28" s="33" t="n">
-        <v>34686</v>
-      </c>
-      <c r="N28" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N28" s="34" t="n">
+        <v/>
       </c>
       <c r="O28" s="35" t="n">
         <v/>
@@ -8189,8 +8241,10 @@
       <c r="CB28" s="48" t="n">
         <v>0.1053232807859264</v>
       </c>
-      <c r="CC28" s="49" t="n">
-        <v>0.1442805039631206</v>
+      <c r="CC28" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="29">
@@ -8208,34 +8262,34 @@
         <v>57929</v>
       </c>
       <c r="D29" s="33" t="n">
-        <v>44.3</v>
+        <v>16.9</v>
       </c>
       <c r="E29" s="33" t="n">
-        <v>25644</v>
+        <v>9804</v>
       </c>
       <c r="F29" s="33" t="n">
-        <v>52.7</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="G29" s="33" t="n">
-        <v>30513</v>
+        <v>48125</v>
       </c>
       <c r="H29" s="33" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="I29" s="33" t="n">
-        <v>389</v>
+        <v>0</v>
       </c>
       <c r="J29" s="33" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="K29" s="33" t="n">
-        <v>1383</v>
+        <v>0</v>
       </c>
       <c r="L29" s="33" t="n">
-        <v>55.7</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="M29" s="33" t="n">
-        <v>32284</v>
+        <v>48125</v>
       </c>
       <c r="N29" s="34" t="inlineStr">
         <is>
@@ -8467,34 +8521,34 @@
         <v>64558</v>
       </c>
       <c r="D30" s="33" t="n">
-        <v>44.3</v>
+        <v>34.7</v>
       </c>
       <c r="E30" s="33" t="n">
-        <v>28579</v>
+        <v>22414</v>
       </c>
       <c r="F30" s="33" t="n">
-        <v>52.7</v>
+        <v>56.9</v>
       </c>
       <c r="G30" s="33" t="n">
-        <v>34004</v>
+        <v>36743</v>
       </c>
       <c r="H30" s="33" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="I30" s="33" t="n">
-        <v>434</v>
+        <v>565</v>
       </c>
       <c r="J30" s="33" t="n">
-        <v>2.4</v>
+        <v>7.5</v>
       </c>
       <c r="K30" s="33" t="n">
-        <v>1541</v>
+        <v>4835</v>
       </c>
       <c r="L30" s="33" t="n">
-        <v>55.7</v>
+        <v>65.3</v>
       </c>
       <c r="M30" s="33" t="n">
-        <v>35979</v>
+        <v>42143</v>
       </c>
       <c r="N30" s="34" t="inlineStr">
         <is>
@@ -8726,34 +8780,34 @@
         <v>78970</v>
       </c>
       <c r="D31" s="33" t="n">
-        <v>44.3</v>
+        <v>40.9</v>
       </c>
       <c r="E31" s="33" t="n">
-        <v>34959</v>
+        <v>32336</v>
       </c>
       <c r="F31" s="33" t="n">
-        <v>52.7</v>
+        <v>58.5</v>
       </c>
       <c r="G31" s="33" t="n">
-        <v>41596</v>
+        <v>46224</v>
       </c>
       <c r="H31" s="33" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="I31" s="33" t="n">
-        <v>531</v>
+        <v>0</v>
       </c>
       <c r="J31" s="33" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
       <c r="K31" s="33" t="n">
-        <v>1885</v>
+        <v>411</v>
       </c>
       <c r="L31" s="33" t="n">
-        <v>55.7</v>
+        <v>59.1</v>
       </c>
       <c r="M31" s="33" t="n">
-        <v>44011</v>
+        <v>46634</v>
       </c>
       <c r="N31" s="34" t="inlineStr">
         <is>
@@ -9019,34 +9073,34 @@
         <v>56103</v>
       </c>
       <c r="D32" s="33" t="n">
-        <v>44.3</v>
+        <v>63</v>
       </c>
       <c r="E32" s="33" t="n">
-        <v>24836</v>
+        <v>35364</v>
       </c>
       <c r="F32" s="33" t="n">
-        <v>52.7</v>
+        <v>36.2</v>
       </c>
       <c r="G32" s="33" t="n">
-        <v>29551</v>
+        <v>20281</v>
       </c>
       <c r="H32" s="33" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I32" s="33" t="n">
-        <v>377</v>
+        <v>458</v>
       </c>
       <c r="J32" s="33" t="n">
-        <v>2.4</v>
+        <v>0</v>
       </c>
       <c r="K32" s="33" t="n">
-        <v>1339</v>
+        <v>0</v>
       </c>
       <c r="L32" s="33" t="n">
-        <v>55.7</v>
+        <v>37</v>
       </c>
       <c r="M32" s="33" t="n">
-        <v>31267</v>
+        <v>20739</v>
       </c>
       <c r="N32" s="34" t="inlineStr">
         <is>
@@ -9278,34 +9332,34 @@
         <v>27419</v>
       </c>
       <c r="D33" s="33" t="n">
-        <v>44.3</v>
+        <v>35.1</v>
       </c>
       <c r="E33" s="33" t="n">
-        <v>12138</v>
+        <v>9622</v>
       </c>
       <c r="F33" s="33" t="n">
-        <v>52.7</v>
+        <v>64.2</v>
       </c>
       <c r="G33" s="33" t="n">
-        <v>14442</v>
+        <v>17601</v>
       </c>
       <c r="H33" s="33" t="n">
-        <v>0.7</v>
+        <v>0.2</v>
       </c>
       <c r="I33" s="33" t="n">
-        <v>184</v>
+        <v>66</v>
       </c>
       <c r="J33" s="33" t="n">
-        <v>2.4</v>
+        <v>0.5</v>
       </c>
       <c r="K33" s="33" t="n">
-        <v>654</v>
+        <v>130</v>
       </c>
       <c r="L33" s="33" t="n">
-        <v>55.7</v>
+        <v>64.90000000000001</v>
       </c>
       <c r="M33" s="33" t="n">
-        <v>15281</v>
+        <v>17797</v>
       </c>
       <c r="N33" s="34" t="inlineStr">
         <is>
@@ -9559,34 +9613,34 @@
         <v>30201</v>
       </c>
       <c r="D34" s="33" t="n">
-        <v>44.3</v>
+        <v>61.8</v>
       </c>
       <c r="E34" s="33" t="n">
-        <v>13369</v>
+        <v>18657</v>
       </c>
       <c r="F34" s="33" t="n">
-        <v>52.7</v>
+        <v>37.1</v>
       </c>
       <c r="G34" s="33" t="n">
-        <v>15908</v>
+        <v>11194</v>
       </c>
       <c r="H34" s="33" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="I34" s="33" t="n">
-        <v>203</v>
+        <v>0</v>
       </c>
       <c r="J34" s="33" t="n">
-        <v>2.4</v>
+        <v>1.2</v>
       </c>
       <c r="K34" s="33" t="n">
-        <v>721</v>
+        <v>349</v>
       </c>
       <c r="L34" s="33" t="n">
-        <v>55.7</v>
+        <v>38.2</v>
       </c>
       <c r="M34" s="33" t="n">
-        <v>16831</v>
+        <v>11544</v>
       </c>
       <c r="N34" s="34" t="inlineStr">
         <is>
@@ -9818,34 +9872,34 @@
         <v>45129</v>
       </c>
       <c r="D35" s="33" t="n">
-        <v>44.3</v>
+        <v>49.5</v>
       </c>
       <c r="E35" s="33" t="n">
-        <v>19978</v>
+        <v>22335</v>
       </c>
       <c r="F35" s="33" t="n">
-        <v>52.7</v>
+        <v>47.8</v>
       </c>
       <c r="G35" s="33" t="n">
-        <v>23771</v>
+        <v>21568</v>
       </c>
       <c r="H35" s="33" t="n">
-        <v>0.7</v>
+        <v>1</v>
       </c>
       <c r="I35" s="33" t="n">
-        <v>303</v>
+        <v>474</v>
       </c>
       <c r="J35" s="33" t="n">
-        <v>2.4</v>
+        <v>1.7</v>
       </c>
       <c r="K35" s="33" t="n">
-        <v>1077</v>
+        <v>753</v>
       </c>
       <c r="L35" s="33" t="n">
-        <v>55.7</v>
+        <v>50.5</v>
       </c>
       <c r="M35" s="33" t="n">
-        <v>25151</v>
+        <v>22794</v>
       </c>
       <c r="N35" s="34" t="inlineStr">
         <is>
@@ -10080,31 +10134,31 @@
         <v>44.3</v>
       </c>
       <c r="E36" s="33" t="n">
-        <v>23993</v>
+        <v>24031</v>
       </c>
       <c r="F36" s="33" t="n">
-        <v>52.7</v>
+        <v>41.3</v>
       </c>
       <c r="G36" s="33" t="n">
-        <v>28548</v>
+        <v>22397</v>
       </c>
       <c r="H36" s="33" t="n">
-        <v>0.7</v>
+        <v>3.4</v>
       </c>
       <c r="I36" s="33" t="n">
-        <v>364</v>
+        <v>1816</v>
       </c>
       <c r="J36" s="33" t="n">
-        <v>2.4</v>
+        <v>11</v>
       </c>
       <c r="K36" s="33" t="n">
-        <v>1294</v>
+        <v>5955</v>
       </c>
       <c r="L36" s="33" t="n">
         <v>55.7</v>
       </c>
       <c r="M36" s="33" t="n">
-        <v>30206</v>
+        <v>30168</v>
       </c>
       <c r="N36" s="34" t="inlineStr">
         <is>
@@ -10336,38 +10390,38 @@
         <v>21460</v>
       </c>
       <c r="D37" s="33" t="n">
-        <v>35.3</v>
+        <v>36.5</v>
       </c>
       <c r="E37" s="33" t="n">
-        <v>7581</v>
+        <v>7841</v>
       </c>
       <c r="F37" s="33" t="n">
-        <v>58.2</v>
+        <v>38.4</v>
       </c>
       <c r="G37" s="33" t="n">
-        <v>12482</v>
+        <v>8241</v>
       </c>
       <c r="H37" s="33" t="n">
-        <v>4.8</v>
+        <v>12.5</v>
       </c>
       <c r="I37" s="33" t="n">
-        <v>1020</v>
+        <v>2686</v>
       </c>
       <c r="J37" s="33" t="n">
-        <v>1.8</v>
+        <v>12.5</v>
       </c>
       <c r="K37" s="33" t="n">
-        <v>377</v>
+        <v>2692</v>
       </c>
       <c r="L37" s="33" t="n">
-        <v>64.7</v>
+        <v>63.5</v>
       </c>
       <c r="M37" s="33" t="n">
-        <v>13879</v>
+        <v>13618</v>
       </c>
       <c r="N37" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O37" s="35" t="n">
@@ -10615,34 +10669,34 @@
         <v>146793</v>
       </c>
       <c r="D38" s="33" t="n">
-        <v>35.3</v>
+        <v>11.7</v>
       </c>
       <c r="E38" s="33" t="n">
-        <v>51854</v>
+        <v>17240</v>
       </c>
       <c r="F38" s="33" t="n">
-        <v>58.2</v>
+        <v>80.2</v>
       </c>
       <c r="G38" s="33" t="n">
-        <v>85384</v>
+        <v>117797</v>
       </c>
       <c r="H38" s="33" t="n">
-        <v>4.8</v>
+        <v>8</v>
       </c>
       <c r="I38" s="33" t="n">
-        <v>6975</v>
+        <v>11756</v>
       </c>
       <c r="J38" s="33" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="K38" s="33" t="n">
-        <v>2580</v>
+        <v>0</v>
       </c>
       <c r="L38" s="33" t="n">
-        <v>64.7</v>
+        <v>88.3</v>
       </c>
       <c r="M38" s="33" t="n">
-        <v>94939</v>
+        <v>129553</v>
       </c>
       <c r="N38" s="34" t="inlineStr">
         <is>
@@ -10874,34 +10928,34 @@
         <v>75398</v>
       </c>
       <c r="D39" s="33" t="n">
-        <v>35.3</v>
+        <v>40.3</v>
       </c>
       <c r="E39" s="33" t="n">
-        <v>26634</v>
+        <v>30410</v>
       </c>
       <c r="F39" s="33" t="n">
-        <v>58.2</v>
+        <v>54.5</v>
       </c>
       <c r="G39" s="33" t="n">
-        <v>43856</v>
+        <v>41074</v>
       </c>
       <c r="H39" s="33" t="n">
-        <v>4.8</v>
+        <v>2.7</v>
       </c>
       <c r="I39" s="33" t="n">
-        <v>3582</v>
+        <v>2006</v>
       </c>
       <c r="J39" s="33" t="n">
-        <v>1.8</v>
+        <v>2.5</v>
       </c>
       <c r="K39" s="33" t="n">
-        <v>1325</v>
+        <v>1907</v>
       </c>
       <c r="L39" s="33" t="n">
-        <v>64.7</v>
+        <v>59.7</v>
       </c>
       <c r="M39" s="33" t="n">
-        <v>48764</v>
+        <v>44988</v>
       </c>
       <c r="N39" s="34" t="inlineStr">
         <is>
@@ -11133,34 +11187,34 @@
         <v>42708</v>
       </c>
       <c r="D40" s="33" t="n">
-        <v>35.3</v>
+        <v>47.6</v>
       </c>
       <c r="E40" s="33" t="n">
-        <v>15086</v>
+        <v>20310</v>
       </c>
       <c r="F40" s="33" t="n">
-        <v>58.2</v>
+        <v>50.2</v>
       </c>
       <c r="G40" s="33" t="n">
-        <v>24842</v>
+        <v>21424</v>
       </c>
       <c r="H40" s="33" t="n">
-        <v>4.8</v>
+        <v>1.7</v>
       </c>
       <c r="I40" s="33" t="n">
-        <v>2029</v>
+        <v>719</v>
       </c>
       <c r="J40" s="33" t="n">
-        <v>1.8</v>
+        <v>0.6</v>
       </c>
       <c r="K40" s="33" t="n">
-        <v>751</v>
+        <v>254</v>
       </c>
       <c r="L40" s="33" t="n">
-        <v>64.7</v>
+        <v>52.4</v>
       </c>
       <c r="M40" s="33" t="n">
-        <v>27621</v>
+        <v>22398</v>
       </c>
       <c r="N40" s="34" t="inlineStr">
         <is>
@@ -11392,34 +11446,34 @@
         <v>71476</v>
       </c>
       <c r="D41" s="33" t="n">
-        <v>35.3</v>
+        <v>59.2</v>
       </c>
       <c r="E41" s="33" t="n">
-        <v>25249</v>
+        <v>42281</v>
       </c>
       <c r="F41" s="33" t="n">
-        <v>58.2</v>
+        <v>37.6</v>
       </c>
       <c r="G41" s="33" t="n">
-        <v>41575</v>
+        <v>26884</v>
       </c>
       <c r="H41" s="33" t="n">
-        <v>4.8</v>
+        <v>1.5</v>
       </c>
       <c r="I41" s="33" t="n">
-        <v>3396</v>
+        <v>1060</v>
       </c>
       <c r="J41" s="33" t="n">
-        <v>1.8</v>
+        <v>1.7</v>
       </c>
       <c r="K41" s="33" t="n">
-        <v>1256</v>
+        <v>1251</v>
       </c>
       <c r="L41" s="33" t="n">
-        <v>64.7</v>
+        <v>40.8</v>
       </c>
       <c r="M41" s="33" t="n">
-        <v>46227</v>
+        <v>29195</v>
       </c>
       <c r="N41" s="34" t="inlineStr">
         <is>
@@ -11687,34 +11741,34 @@
         <v>16850</v>
       </c>
       <c r="D42" s="33" t="n">
-        <v>36.4</v>
+        <v>76.7</v>
       </c>
       <c r="E42" s="33" t="n">
-        <v>6141</v>
+        <v>12931</v>
       </c>
       <c r="F42" s="33" t="n">
-        <v>57</v>
+        <v>22.1</v>
       </c>
       <c r="G42" s="33" t="n">
-        <v>9606</v>
+        <v>3730</v>
       </c>
       <c r="H42" s="33" t="n">
-        <v>4.4</v>
+        <v>0.5</v>
       </c>
       <c r="I42" s="33" t="n">
-        <v>741</v>
+        <v>91</v>
       </c>
       <c r="J42" s="33" t="n">
-        <v>2.1</v>
+        <v>0.6</v>
       </c>
       <c r="K42" s="33" t="n">
-        <v>362</v>
+        <v>97</v>
       </c>
       <c r="L42" s="33" t="n">
-        <v>63.6</v>
+        <v>23.3</v>
       </c>
       <c r="M42" s="33" t="n">
-        <v>10709</v>
+        <v>3918</v>
       </c>
       <c r="N42" s="34" t="inlineStr">
         <is>
@@ -11946,34 +12000,34 @@
         <v>24227</v>
       </c>
       <c r="D43" s="33" t="n">
-        <v>36.4</v>
+        <v>39.1</v>
       </c>
       <c r="E43" s="33" t="n">
-        <v>8830</v>
+        <v>9467</v>
       </c>
       <c r="F43" s="33" t="n">
-        <v>57</v>
+        <v>56.1</v>
       </c>
       <c r="G43" s="33" t="n">
-        <v>13812</v>
+        <v>13598</v>
       </c>
       <c r="H43" s="33" t="n">
-        <v>4.4</v>
+        <v>4.3</v>
       </c>
       <c r="I43" s="33" t="n">
-        <v>1065</v>
+        <v>1040</v>
       </c>
       <c r="J43" s="33" t="n">
-        <v>2.1</v>
+        <v>0.5</v>
       </c>
       <c r="K43" s="33" t="n">
-        <v>521</v>
+        <v>122</v>
       </c>
       <c r="L43" s="33" t="n">
-        <v>63.6</v>
+        <v>60.9</v>
       </c>
       <c r="M43" s="33" t="n">
-        <v>15398</v>
+        <v>14760</v>
       </c>
       <c r="N43" s="34" t="inlineStr">
         <is>
@@ -12202,42 +12256,40 @@
         </is>
       </c>
       <c r="C44" s="33" t="n">
-        <v>33969</v>
+        <v/>
       </c>
       <c r="D44" s="33" t="n">
-        <v>36.4</v>
+        <v/>
       </c>
       <c r="E44" s="33" t="n">
-        <v>12380</v>
+        <v/>
       </c>
       <c r="F44" s="33" t="n">
-        <v>57</v>
+        <v/>
       </c>
       <c r="G44" s="33" t="n">
-        <v>19366</v>
+        <v/>
       </c>
       <c r="H44" s="33" t="n">
-        <v>4.4</v>
+        <v/>
       </c>
       <c r="I44" s="33" t="n">
-        <v>1493</v>
+        <v/>
       </c>
       <c r="J44" s="33" t="n">
-        <v>2.1</v>
+        <v/>
       </c>
       <c r="K44" s="33" t="n">
-        <v>730</v>
+        <v/>
       </c>
       <c r="L44" s="33" t="n">
-        <v>63.6</v>
+        <v/>
       </c>
       <c r="M44" s="33" t="n">
-        <v>21589</v>
-      </c>
-      <c r="N44" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N44" s="34" t="n">
+        <v/>
       </c>
       <c r="O44" s="35" t="n">
         <v/>
@@ -12445,8 +12497,10 @@
       <c r="CB44" s="48" t="n">
         <v>0.2620501420974141</v>
       </c>
-      <c r="CC44" s="49" t="n">
-        <v>0.3429432302970201</v>
+      <c r="CC44" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="45">
@@ -12464,34 +12518,34 @@
         <v>27037</v>
       </c>
       <c r="D45" s="33" t="n">
-        <v>36.4</v>
+        <v>44.1</v>
       </c>
       <c r="E45" s="33" t="n">
-        <v>9854</v>
+        <v>11926</v>
       </c>
       <c r="F45" s="33" t="n">
-        <v>57</v>
+        <v>51.5</v>
       </c>
       <c r="G45" s="33" t="n">
-        <v>15414</v>
+        <v>13913</v>
       </c>
       <c r="H45" s="33" t="n">
-        <v>4.4</v>
+        <v>1.9</v>
       </c>
       <c r="I45" s="33" t="n">
-        <v>1188</v>
+        <v>517</v>
       </c>
       <c r="J45" s="33" t="n">
-        <v>2.1</v>
+        <v>2.5</v>
       </c>
       <c r="K45" s="33" t="n">
-        <v>581</v>
+        <v>682</v>
       </c>
       <c r="L45" s="33" t="n">
-        <v>63.6</v>
+        <v>55.9</v>
       </c>
       <c r="M45" s="33" t="n">
-        <v>17184</v>
+        <v>15111</v>
       </c>
       <c r="N45" s="34" t="inlineStr">
         <is>
@@ -12720,42 +12774,40 @@
         </is>
       </c>
       <c r="C46" s="33" t="n">
-        <v>24991</v>
+        <v/>
       </c>
       <c r="D46" s="33" t="n">
-        <v>36.4</v>
+        <v/>
       </c>
       <c r="E46" s="33" t="n">
-        <v>9108</v>
+        <v/>
       </c>
       <c r="F46" s="33" t="n">
-        <v>57</v>
+        <v/>
       </c>
       <c r="G46" s="33" t="n">
-        <v>14248</v>
+        <v/>
       </c>
       <c r="H46" s="33" t="n">
-        <v>4.4</v>
+        <v/>
       </c>
       <c r="I46" s="33" t="n">
-        <v>1098</v>
+        <v/>
       </c>
       <c r="J46" s="33" t="n">
-        <v>2.1</v>
+        <v/>
       </c>
       <c r="K46" s="33" t="n">
-        <v>537</v>
+        <v/>
       </c>
       <c r="L46" s="33" t="n">
-        <v>63.6</v>
+        <v/>
       </c>
       <c r="M46" s="33" t="n">
-        <v>15883</v>
-      </c>
-      <c r="N46" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N46" s="34" t="n">
+        <v/>
       </c>
       <c r="O46" s="35" t="n">
         <v/>
@@ -12963,8 +13015,10 @@
       <c r="CB46" s="48" t="n">
         <v>0.4060030935161574</v>
       </c>
-      <c r="CC46" s="49" t="n">
-        <v>0.4594156744166978</v>
+      <c r="CC46" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="47">
@@ -12982,38 +13036,38 @@
         <v>53111</v>
       </c>
       <c r="D47" s="33" t="n">
-        <v>36.4</v>
+        <v>15.7</v>
       </c>
       <c r="E47" s="33" t="n">
-        <v>19356</v>
+        <v>8324</v>
       </c>
       <c r="F47" s="33" t="n">
-        <v>57</v>
+        <v>63.1</v>
       </c>
       <c r="G47" s="33" t="n">
-        <v>30279</v>
+        <v>33517</v>
       </c>
       <c r="H47" s="33" t="n">
-        <v>4.4</v>
+        <v>11.7</v>
       </c>
       <c r="I47" s="33" t="n">
-        <v>2334</v>
+        <v>6234</v>
       </c>
       <c r="J47" s="33" t="n">
-        <v>2.1</v>
+        <v>9.5</v>
       </c>
       <c r="K47" s="33" t="n">
-        <v>1141</v>
+        <v>5037</v>
       </c>
       <c r="L47" s="33" t="n">
-        <v>63.6</v>
+        <v>84.3</v>
       </c>
       <c r="M47" s="33" t="n">
-        <v>33755</v>
+        <v>44788</v>
       </c>
       <c r="N47" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="O47" s="35" t="n">
@@ -13238,42 +13292,40 @@
         </is>
       </c>
       <c r="C48" s="33" t="n">
-        <v>46284</v>
+        <v/>
       </c>
       <c r="D48" s="33" t="n">
-        <v>36.4</v>
+        <v/>
       </c>
       <c r="E48" s="33" t="n">
-        <v>16868</v>
+        <v/>
       </c>
       <c r="F48" s="33" t="n">
-        <v>57</v>
+        <v/>
       </c>
       <c r="G48" s="33" t="n">
-        <v>26387</v>
+        <v/>
       </c>
       <c r="H48" s="33" t="n">
-        <v>4.4</v>
+        <v/>
       </c>
       <c r="I48" s="33" t="n">
-        <v>2034</v>
+        <v/>
       </c>
       <c r="J48" s="33" t="n">
-        <v>2.1</v>
+        <v/>
       </c>
       <c r="K48" s="33" t="n">
-        <v>995</v>
+        <v/>
       </c>
       <c r="L48" s="33" t="n">
-        <v>63.6</v>
+        <v/>
       </c>
       <c r="M48" s="33" t="n">
-        <v>29416</v>
-      </c>
-      <c r="N48" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N48" s="34" t="n">
+        <v/>
       </c>
       <c r="O48" s="35" t="n">
         <v/>
@@ -13481,8 +13533,10 @@
       <c r="CB48" s="48" t="n">
         <v>0.2556860130034057</v>
       </c>
-      <c r="CC48" s="49" t="n">
-        <v>0.5548019956342074</v>
+      <c r="CC48" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="49">
@@ -13497,42 +13551,40 @@
         </is>
       </c>
       <c r="C49" s="33" t="n">
-        <v>37799</v>
+        <v/>
       </c>
       <c r="D49" s="33" t="n">
-        <v>36.4</v>
+        <v/>
       </c>
       <c r="E49" s="33" t="n">
-        <v>13776</v>
+        <v/>
       </c>
       <c r="F49" s="33" t="n">
-        <v>57</v>
+        <v/>
       </c>
       <c r="G49" s="33" t="n">
-        <v>21550</v>
+        <v/>
       </c>
       <c r="H49" s="33" t="n">
-        <v>4.4</v>
+        <v/>
       </c>
       <c r="I49" s="33" t="n">
-        <v>1661</v>
+        <v/>
       </c>
       <c r="J49" s="33" t="n">
-        <v>2.1</v>
+        <v/>
       </c>
       <c r="K49" s="33" t="n">
-        <v>812</v>
+        <v/>
       </c>
       <c r="L49" s="33" t="n">
-        <v>63.6</v>
+        <v/>
       </c>
       <c r="M49" s="33" t="n">
-        <v>24024</v>
-      </c>
-      <c r="N49" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N49" s="34" t="n">
+        <v/>
       </c>
       <c r="O49" s="35" t="n">
         <v/>
@@ -13740,8 +13792,10 @@
       <c r="CB49" s="48" t="n">
         <v>0.08937584328619259</v>
       </c>
-      <c r="CC49" s="49" t="n">
-        <v>0.1092694936068901</v>
+      <c r="CC49" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="50">
@@ -13759,34 +13813,34 @@
         <v>122957</v>
       </c>
       <c r="D50" s="33" t="n">
-        <v>36.4</v>
+        <v>16.1</v>
       </c>
       <c r="E50" s="33" t="n">
-        <v>44811</v>
+        <v>19830</v>
       </c>
       <c r="F50" s="33" t="n">
-        <v>57</v>
+        <v>83.7</v>
       </c>
       <c r="G50" s="33" t="n">
-        <v>70099</v>
+        <v>102905</v>
       </c>
       <c r="H50" s="33" t="n">
-        <v>4.4</v>
+        <v>0</v>
       </c>
       <c r="I50" s="33" t="n">
-        <v>5405</v>
+        <v>37</v>
       </c>
       <c r="J50" s="33" t="n">
-        <v>2.1</v>
+        <v>0.2</v>
       </c>
       <c r="K50" s="33" t="n">
-        <v>2642</v>
+        <v>186</v>
       </c>
       <c r="L50" s="33" t="n">
-        <v>63.6</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="M50" s="33" t="n">
-        <v>78146</v>
+        <v>103128</v>
       </c>
       <c r="N50" s="34" t="inlineStr">
         <is>
@@ -14018,38 +14072,38 @@
         <v>23691</v>
       </c>
       <c r="D51" s="33" t="n">
-        <v>34.5</v>
+        <v>83.2</v>
       </c>
       <c r="E51" s="33" t="n">
-        <v>8171</v>
+        <v>19715</v>
       </c>
       <c r="F51" s="33" t="n">
-        <v>45.1</v>
+        <v>16.8</v>
       </c>
       <c r="G51" s="33" t="n">
-        <v>10676</v>
+        <v>3977</v>
       </c>
       <c r="H51" s="33" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I51" s="33" t="n">
-        <v>1174</v>
+        <v>0</v>
       </c>
       <c r="J51" s="33" t="n">
-        <v>15.5</v>
+        <v>0</v>
       </c>
       <c r="K51" s="33" t="n">
-        <v>3670</v>
+        <v>0</v>
       </c>
       <c r="L51" s="33" t="n">
-        <v>65.5</v>
+        <v>16.8</v>
       </c>
       <c r="M51" s="33" t="n">
-        <v>15520</v>
+        <v>3977</v>
       </c>
       <c r="N51" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="O51" s="35" t="n">
@@ -14277,34 +14331,34 @@
         <v>32052</v>
       </c>
       <c r="D52" s="33" t="n">
-        <v>34.5</v>
+        <v>4.2</v>
       </c>
       <c r="E52" s="33" t="n">
-        <v>11055</v>
+        <v>1336</v>
       </c>
       <c r="F52" s="33" t="n">
-        <v>45.1</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G52" s="33" t="n">
-        <v>14444</v>
+        <v>2671</v>
       </c>
       <c r="H52" s="33" t="n">
-        <v>5</v>
+        <v>87.5</v>
       </c>
       <c r="I52" s="33" t="n">
-        <v>1589</v>
+        <v>28046</v>
       </c>
       <c r="J52" s="33" t="n">
-        <v>15.5</v>
+        <v>0</v>
       </c>
       <c r="K52" s="33" t="n">
-        <v>4965</v>
+        <v>0</v>
       </c>
       <c r="L52" s="33" t="n">
-        <v>65.5</v>
+        <v>95.8</v>
       </c>
       <c r="M52" s="33" t="n">
-        <v>20997</v>
+        <v>30717</v>
       </c>
       <c r="N52" s="34" t="inlineStr">
         <is>
@@ -14536,38 +14590,38 @@
         <v>23092</v>
       </c>
       <c r="D53" s="33" t="n">
-        <v>34.5</v>
+        <v>1.7</v>
       </c>
       <c r="E53" s="33" t="n">
-        <v>7965</v>
+        <v>399</v>
       </c>
       <c r="F53" s="33" t="n">
-        <v>45.1</v>
+        <v>77.8</v>
       </c>
       <c r="G53" s="33" t="n">
-        <v>10406</v>
+        <v>17965</v>
       </c>
       <c r="H53" s="33" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="I53" s="33" t="n">
-        <v>1145</v>
+        <v>0</v>
       </c>
       <c r="J53" s="33" t="n">
-        <v>15.5</v>
+        <v>20.5</v>
       </c>
       <c r="K53" s="33" t="n">
-        <v>3577</v>
+        <v>4728</v>
       </c>
       <c r="L53" s="33" t="n">
-        <v>65.5</v>
+        <v>98.3</v>
       </c>
       <c r="M53" s="33" t="n">
-        <v>15127</v>
+        <v>22693</v>
       </c>
       <c r="N53" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O53" s="35" t="n">
@@ -14792,42 +14846,40 @@
         </is>
       </c>
       <c r="C54" s="33" t="n">
-        <v>102222</v>
+        <v/>
       </c>
       <c r="D54" s="33" t="n">
-        <v>34.5</v>
+        <v/>
       </c>
       <c r="E54" s="33" t="n">
-        <v>35257</v>
+        <v/>
       </c>
       <c r="F54" s="33" t="n">
-        <v>45.1</v>
+        <v/>
       </c>
       <c r="G54" s="33" t="n">
-        <v>46064</v>
+        <v/>
       </c>
       <c r="H54" s="33" t="n">
-        <v>5</v>
+        <v/>
       </c>
       <c r="I54" s="33" t="n">
-        <v>5067</v>
+        <v/>
       </c>
       <c r="J54" s="33" t="n">
-        <v>15.5</v>
+        <v/>
       </c>
       <c r="K54" s="33" t="n">
-        <v>15834</v>
+        <v/>
       </c>
       <c r="L54" s="33" t="n">
-        <v>65.5</v>
+        <v/>
       </c>
       <c r="M54" s="33" t="n">
-        <v>66964</v>
-      </c>
-      <c r="N54" s="34" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N54" s="34" t="n">
+        <v/>
       </c>
       <c r="O54" s="35" t="n">
         <v/>
@@ -15055,8 +15107,10 @@
       <c r="CB54" s="48" t="n">
         <v>0.0106654677979396</v>
       </c>
-      <c r="CC54" s="49" t="n">
-        <v>0.05996060344215216</v>
+      <c r="CC54" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="55">
@@ -15074,38 +15128,38 @@
         <v>37266</v>
       </c>
       <c r="D55" s="33" t="n">
-        <v>34.5</v>
+        <v>16.3</v>
       </c>
       <c r="E55" s="33" t="n">
-        <v>12853</v>
+        <v>6087</v>
       </c>
       <c r="F55" s="33" t="n">
-        <v>45.1</v>
+        <v>33.4</v>
       </c>
       <c r="G55" s="33" t="n">
-        <v>16793</v>
+        <v>12447</v>
       </c>
       <c r="H55" s="33" t="n">
-        <v>5</v>
+        <v>7.1</v>
       </c>
       <c r="I55" s="33" t="n">
-        <v>1847</v>
+        <v>2638</v>
       </c>
       <c r="J55" s="33" t="n">
-        <v>15.5</v>
+        <v>43.2</v>
       </c>
       <c r="K55" s="33" t="n">
-        <v>5772</v>
+        <v>16093</v>
       </c>
       <c r="L55" s="33" t="n">
-        <v>65.5</v>
+        <v>83.7</v>
       </c>
       <c r="M55" s="33" t="n">
-        <v>24412</v>
+        <v>31178</v>
       </c>
       <c r="N55" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O55" s="35" t="n">
@@ -15333,38 +15387,38 @@
         <v>36768</v>
       </c>
       <c r="D56" s="33" t="n">
-        <v>34.5</v>
+        <v>38.8</v>
       </c>
       <c r="E56" s="33" t="n">
-        <v>12682</v>
+        <v>14284</v>
       </c>
       <c r="F56" s="33" t="n">
-        <v>45.1</v>
+        <v>42.5</v>
       </c>
       <c r="G56" s="33" t="n">
-        <v>16569</v>
+        <v>15614</v>
       </c>
       <c r="H56" s="33" t="n">
-        <v>5</v>
+        <v>11.5</v>
       </c>
       <c r="I56" s="33" t="n">
-        <v>1822</v>
+        <v>4234</v>
       </c>
       <c r="J56" s="33" t="n">
-        <v>15.5</v>
+        <v>7.2</v>
       </c>
       <c r="K56" s="33" t="n">
-        <v>5695</v>
+        <v>2636</v>
       </c>
       <c r="L56" s="33" t="n">
-        <v>65.5</v>
+        <v>61.2</v>
       </c>
       <c r="M56" s="33" t="n">
-        <v>24086</v>
+        <v>22484</v>
       </c>
       <c r="N56" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O56" s="35" t="n">
@@ -15592,38 +15646,38 @@
         <v>38747</v>
       </c>
       <c r="D57" s="33" t="n">
-        <v>34.5</v>
+        <v>82.40000000000001</v>
       </c>
       <c r="E57" s="33" t="n">
-        <v>13364</v>
+        <v>31909</v>
       </c>
       <c r="F57" s="33" t="n">
-        <v>45.1</v>
+        <v>14.2</v>
       </c>
       <c r="G57" s="33" t="n">
-        <v>17460</v>
+        <v>5513</v>
       </c>
       <c r="H57" s="33" t="n">
-        <v>5</v>
+        <v>3.4</v>
       </c>
       <c r="I57" s="33" t="n">
-        <v>1920</v>
+        <v>1318</v>
       </c>
       <c r="J57" s="33" t="n">
-        <v>15.5</v>
+        <v>0</v>
       </c>
       <c r="K57" s="33" t="n">
-        <v>6002</v>
+        <v>7</v>
       </c>
       <c r="L57" s="33" t="n">
-        <v>65.5</v>
+        <v>17.6</v>
       </c>
       <c r="M57" s="33" t="n">
-        <v>25383</v>
+        <v>6838</v>
       </c>
       <c r="N57" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="O57" s="35" t="n">
@@ -15867,38 +15921,38 @@
         <v>21620</v>
       </c>
       <c r="D58" s="33" t="n">
-        <v>34.5</v>
+        <v>50.3</v>
       </c>
       <c r="E58" s="33" t="n">
-        <v>7457</v>
+        <v>10866</v>
       </c>
       <c r="F58" s="33" t="n">
-        <v>45.1</v>
+        <v>29.9</v>
       </c>
       <c r="G58" s="33" t="n">
-        <v>9743</v>
+        <v>6454</v>
       </c>
       <c r="H58" s="33" t="n">
-        <v>5</v>
+        <v>16.6</v>
       </c>
       <c r="I58" s="33" t="n">
-        <v>1072</v>
+        <v>3583</v>
       </c>
       <c r="J58" s="33" t="n">
-        <v>15.5</v>
+        <v>3.3</v>
       </c>
       <c r="K58" s="33" t="n">
-        <v>3349</v>
+        <v>718</v>
       </c>
       <c r="L58" s="33" t="n">
-        <v>65.5</v>
+        <v>49.7</v>
       </c>
       <c r="M58" s="33" t="n">
-        <v>14163</v>
+        <v>10755</v>
       </c>
       <c r="N58" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O58" s="35" t="n">
@@ -16126,38 +16180,38 @@
         <v>49163</v>
       </c>
       <c r="D59" s="33" t="n">
-        <v>34.5</v>
+        <v>48.1</v>
       </c>
       <c r="E59" s="33" t="n">
-        <v>16957</v>
+        <v>23651</v>
       </c>
       <c r="F59" s="33" t="n">
-        <v>45.1</v>
+        <v>40.2</v>
       </c>
       <c r="G59" s="33" t="n">
-        <v>22154</v>
+        <v>19782</v>
       </c>
       <c r="H59" s="33" t="n">
-        <v>5</v>
+        <v>4.9</v>
       </c>
       <c r="I59" s="33" t="n">
-        <v>2437</v>
+        <v>2396</v>
       </c>
       <c r="J59" s="33" t="n">
-        <v>15.5</v>
+        <v>6.8</v>
       </c>
       <c r="K59" s="33" t="n">
-        <v>7615</v>
+        <v>3334</v>
       </c>
       <c r="L59" s="33" t="n">
-        <v>65.5</v>
+        <v>51.9</v>
       </c>
       <c r="M59" s="33" t="n">
-        <v>32206</v>
+        <v>25512</v>
       </c>
       <c r="N59" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O59" s="35" t="n">
@@ -16385,38 +16439,38 @@
         <v>10650</v>
       </c>
       <c r="D60" s="33" t="n">
-        <v>34.5</v>
+        <v>52.2</v>
       </c>
       <c r="E60" s="33" t="n">
-        <v>3673</v>
+        <v>5559</v>
       </c>
       <c r="F60" s="33" t="n">
-        <v>45.1</v>
+        <v>37.1</v>
       </c>
       <c r="G60" s="33" t="n">
-        <v>4799</v>
+        <v>3956</v>
       </c>
       <c r="H60" s="33" t="n">
-        <v>5</v>
+        <v>2.5</v>
       </c>
       <c r="I60" s="33" t="n">
-        <v>528</v>
+        <v>270</v>
       </c>
       <c r="J60" s="33" t="n">
-        <v>15.5</v>
+        <v>8.1</v>
       </c>
       <c r="K60" s="33" t="n">
-        <v>1650</v>
+        <v>865</v>
       </c>
       <c r="L60" s="33" t="n">
-        <v>65.5</v>
+        <v>47.8</v>
       </c>
       <c r="M60" s="33" t="n">
-        <v>6977</v>
+        <v>5091</v>
       </c>
       <c r="N60" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O60" s="35" t="n">
@@ -16644,38 +16698,38 @@
         <v>229301</v>
       </c>
       <c r="D61" s="33" t="n">
-        <v>34.5</v>
+        <v>54.9</v>
       </c>
       <c r="E61" s="33" t="n">
-        <v>79089</v>
+        <v>125972</v>
       </c>
       <c r="F61" s="33" t="n">
+        <v>43.2</v>
+      </c>
+      <c r="G61" s="33" t="n">
+        <v>99116</v>
+      </c>
+      <c r="H61" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="I61" s="33" t="n">
+        <v>0</v>
+      </c>
+      <c r="J61" s="33" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="K61" s="33" t="n">
+        <v>4213</v>
+      </c>
+      <c r="L61" s="33" t="n">
         <v>45.1</v>
       </c>
-      <c r="G61" s="33" t="n">
-        <v>103330</v>
-      </c>
-      <c r="H61" s="33" t="n">
-        <v>5</v>
-      </c>
-      <c r="I61" s="33" t="n">
-        <v>11365</v>
-      </c>
-      <c r="J61" s="33" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="K61" s="33" t="n">
-        <v>35517</v>
-      </c>
-      <c r="L61" s="33" t="n">
-        <v>65.5</v>
-      </c>
       <c r="M61" s="33" t="n">
-        <v>150212</v>
+        <v>103329</v>
       </c>
       <c r="N61" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="O61" s="35" t="n">
@@ -16903,38 +16957,38 @@
         <v>48802</v>
       </c>
       <c r="D62" s="33" t="n">
-        <v>34.5</v>
+        <v>12.2</v>
       </c>
       <c r="E62" s="33" t="n">
-        <v>16832</v>
+        <v>5940</v>
       </c>
       <c r="F62" s="33" t="n">
-        <v>45.1</v>
+        <v>32.9</v>
       </c>
       <c r="G62" s="33" t="n">
-        <v>21992</v>
+        <v>16064</v>
       </c>
       <c r="H62" s="33" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="I62" s="33" t="n">
-        <v>2419</v>
+        <v>2927</v>
       </c>
       <c r="J62" s="33" t="n">
-        <v>15.5</v>
+        <v>48.9</v>
       </c>
       <c r="K62" s="33" t="n">
-        <v>7559</v>
+        <v>23871</v>
       </c>
       <c r="L62" s="33" t="n">
-        <v>65.5</v>
+        <v>87.8</v>
       </c>
       <c r="M62" s="33" t="n">
-        <v>31970</v>
+        <v>42862</v>
       </c>
       <c r="N62" s="34" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O62" s="35" t="n">
@@ -17159,42 +17213,40 @@
         </is>
       </c>
       <c r="C63" s="33" t="n">
-        <v>45078</v>
+        <v/>
       </c>
       <c r="D63" s="33" t="n">
-        <v>43.6</v>
+        <v/>
       </c>
       <c r="E63" s="33" t="n">
-        <v>19634</v>
+        <v/>
       </c>
       <c r="F63" s="33" t="n">
-        <v>52.4</v>
+        <v/>
       </c>
       <c r="G63" s="33" t="n">
-        <v>23610</v>
+        <v/>
       </c>
       <c r="H63" s="33" t="n">
-        <v>1.1</v>
+        <v/>
       </c>
       <c r="I63" s="33" t="n">
-        <v>509</v>
+        <v/>
       </c>
       <c r="J63" s="33" t="n">
-        <v>2.9</v>
+        <v/>
       </c>
       <c r="K63" s="33" t="n">
-        <v>1325</v>
+        <v/>
       </c>
       <c r="L63" s="33" t="n">
-        <v>56.4</v>
+        <v/>
       </c>
       <c r="M63" s="33" t="n">
-        <v>25444</v>
-      </c>
-      <c r="N63" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N63" s="34" t="n">
+        <v/>
       </c>
       <c r="O63" s="35" t="n">
         <v/>
@@ -17402,8 +17454,10 @@
       <c r="CB63" s="48" t="n">
         <v>0.1135861167241174</v>
       </c>
-      <c r="CC63" s="49" t="n">
-        <v>0.1530251853324076</v>
+      <c r="CC63" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="64">
@@ -17421,34 +17475,34 @@
         <v>121379</v>
       </c>
       <c r="D64" s="33" t="n">
-        <v>43.6</v>
+        <v>44.1</v>
       </c>
       <c r="E64" s="33" t="n">
-        <v>52868</v>
+        <v>53567</v>
       </c>
       <c r="F64" s="33" t="n">
-        <v>52.4</v>
+        <v>55.9</v>
       </c>
       <c r="G64" s="33" t="n">
-        <v>63572</v>
+        <v>67812</v>
       </c>
       <c r="H64" s="33" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="I64" s="33" t="n">
-        <v>1370</v>
+        <v>0</v>
       </c>
       <c r="J64" s="33" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
       <c r="K64" s="33" t="n">
-        <v>3569</v>
+        <v>0</v>
       </c>
       <c r="L64" s="33" t="n">
-        <v>56.4</v>
+        <v>55.9</v>
       </c>
       <c r="M64" s="33" t="n">
-        <v>68511</v>
+        <v>67812</v>
       </c>
       <c r="N64" s="34" t="inlineStr">
         <is>
@@ -17680,34 +17734,34 @@
         <v>65217</v>
       </c>
       <c r="D65" s="33" t="n">
-        <v>43.6</v>
+        <v>19.7</v>
       </c>
       <c r="E65" s="33" t="n">
-        <v>28406</v>
+        <v>12830</v>
       </c>
       <c r="F65" s="33" t="n">
-        <v>52.4</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="G65" s="33" t="n">
-        <v>34157</v>
+        <v>48015</v>
       </c>
       <c r="H65" s="33" t="n">
-        <v>1.1</v>
+        <v>3.6</v>
       </c>
       <c r="I65" s="33" t="n">
-        <v>736</v>
+        <v>2375</v>
       </c>
       <c r="J65" s="33" t="n">
-        <v>2.9</v>
+        <v>3.1</v>
       </c>
       <c r="K65" s="33" t="n">
-        <v>1918</v>
+        <v>1997</v>
       </c>
       <c r="L65" s="33" t="n">
-        <v>56.4</v>
+        <v>80.3</v>
       </c>
       <c r="M65" s="33" t="n">
-        <v>36811</v>
+        <v>52387</v>
       </c>
       <c r="N65" s="34" t="inlineStr">
         <is>
@@ -17939,34 +17993,34 @@
         <v>79932</v>
       </c>
       <c r="D66" s="33" t="n">
-        <v>43.6</v>
+        <v>25.1</v>
       </c>
       <c r="E66" s="33" t="n">
-        <v>34815</v>
+        <v>20069</v>
       </c>
       <c r="F66" s="33" t="n">
-        <v>52.4</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="G66" s="33" t="n">
-        <v>41864</v>
+        <v>56428</v>
       </c>
       <c r="H66" s="33" t="n">
-        <v>1.1</v>
+        <v>2</v>
       </c>
       <c r="I66" s="33" t="n">
-        <v>902</v>
+        <v>1566</v>
       </c>
       <c r="J66" s="33" t="n">
-        <v>2.9</v>
+        <v>2.3</v>
       </c>
       <c r="K66" s="33" t="n">
-        <v>2350</v>
+        <v>1869</v>
       </c>
       <c r="L66" s="33" t="n">
-        <v>56.4</v>
+        <v>74.90000000000001</v>
       </c>
       <c r="M66" s="33" t="n">
-        <v>45117</v>
+        <v>59863</v>
       </c>
       <c r="N66" s="34" t="inlineStr">
         <is>
@@ -18198,34 +18252,34 @@
         <v>38972</v>
       </c>
       <c r="D67" s="33" t="n">
-        <v>43.6</v>
+        <v>59.5</v>
       </c>
       <c r="E67" s="33" t="n">
-        <v>16975</v>
+        <v>23179</v>
       </c>
       <c r="F67" s="33" t="n">
-        <v>52.4</v>
+        <v>40.5</v>
       </c>
       <c r="G67" s="33" t="n">
-        <v>20411</v>
+        <v>15793</v>
       </c>
       <c r="H67" s="33" t="n">
-        <v>1.1</v>
+        <v>0</v>
       </c>
       <c r="I67" s="33" t="n">
-        <v>440</v>
+        <v>0</v>
       </c>
       <c r="J67" s="33" t="n">
-        <v>2.9</v>
+        <v>0</v>
       </c>
       <c r="K67" s="33" t="n">
-        <v>1146</v>
+        <v>0</v>
       </c>
       <c r="L67" s="33" t="n">
-        <v>56.4</v>
+        <v>40.5</v>
       </c>
       <c r="M67" s="33" t="n">
-        <v>21997</v>
+        <v>15793</v>
       </c>
       <c r="N67" s="34" t="inlineStr">
         <is>
@@ -18457,34 +18511,34 @@
         <v>120980</v>
       </c>
       <c r="D68" s="33" t="n">
-        <v>43.6</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="E68" s="33" t="n">
-        <v>52694</v>
+        <v>85758</v>
       </c>
       <c r="F68" s="33" t="n">
-        <v>52.4</v>
+        <v>20.7</v>
       </c>
       <c r="G68" s="33" t="n">
-        <v>63363</v>
+        <v>24997</v>
       </c>
       <c r="H68" s="33" t="n">
-        <v>1.1</v>
+        <v>0.4</v>
       </c>
       <c r="I68" s="33" t="n">
-        <v>1366</v>
+        <v>494</v>
       </c>
       <c r="J68" s="33" t="n">
-        <v>2.9</v>
+        <v>8</v>
       </c>
       <c r="K68" s="33" t="n">
-        <v>3557</v>
+        <v>9731</v>
       </c>
       <c r="L68" s="33" t="n">
-        <v>56.4</v>
+        <v>29.1</v>
       </c>
       <c r="M68" s="33" t="n">
-        <v>68286</v>
+        <v>35222</v>
       </c>
       <c r="N68" s="34" t="inlineStr">
         <is>
@@ -18752,34 +18806,34 @@
         <v>97232</v>
       </c>
       <c r="D69" s="33" t="n">
-        <v>52.9</v>
+        <v>48.3</v>
       </c>
       <c r="E69" s="33" t="n">
-        <v>51431</v>
+        <v>46971</v>
       </c>
       <c r="F69" s="33" t="n">
-        <v>39.4</v>
+        <v>48.5</v>
       </c>
       <c r="G69" s="33" t="n">
-        <v>38322</v>
+        <v>47113</v>
       </c>
       <c r="H69" s="33" t="n">
-        <v>0.7</v>
+        <v>0.8</v>
       </c>
       <c r="I69" s="33" t="n">
-        <v>700</v>
+        <v>752</v>
       </c>
       <c r="J69" s="33" t="n">
-        <v>7</v>
+        <v>2.5</v>
       </c>
       <c r="K69" s="33" t="n">
-        <v>6780</v>
+        <v>2395</v>
       </c>
       <c r="L69" s="33" t="n">
-        <v>47.1</v>
+        <v>51.7</v>
       </c>
       <c r="M69" s="33" t="n">
-        <v>45801</v>
+        <v>50260</v>
       </c>
       <c r="N69" s="34" t="inlineStr">
         <is>
@@ -19011,34 +19065,34 @@
         <v>28327</v>
       </c>
       <c r="D70" s="33" t="n">
-        <v>52.9</v>
+        <v>31.9</v>
       </c>
       <c r="E70" s="33" t="n">
-        <v>14984</v>
+        <v>9043</v>
       </c>
       <c r="F70" s="33" t="n">
-        <v>39.4</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="G70" s="33" t="n">
-        <v>11165</v>
+        <v>19284</v>
       </c>
       <c r="H70" s="33" t="n">
-        <v>0.7</v>
+        <v>0</v>
       </c>
       <c r="I70" s="33" t="n">
-        <v>204</v>
+        <v>0</v>
       </c>
       <c r="J70" s="33" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="K70" s="33" t="n">
-        <v>1975</v>
+        <v>0</v>
       </c>
       <c r="L70" s="33" t="n">
-        <v>47.1</v>
+        <v>68.09999999999999</v>
       </c>
       <c r="M70" s="33" t="n">
-        <v>13344</v>
+        <v>19284</v>
       </c>
       <c r="N70" s="34" t="inlineStr">
         <is>
@@ -19270,34 +19324,34 @@
         <v>90464</v>
       </c>
       <c r="D71" s="33" t="n">
-        <v>52.9</v>
+        <v>56.1</v>
       </c>
       <c r="E71" s="33" t="n">
-        <v>47851</v>
+        <v>50736</v>
       </c>
       <c r="F71" s="33" t="n">
-        <v>39.4</v>
+        <v>33.6</v>
       </c>
       <c r="G71" s="33" t="n">
-        <v>35654</v>
+        <v>30436</v>
       </c>
       <c r="H71" s="33" t="n">
         <v>0.7</v>
       </c>
       <c r="I71" s="33" t="n">
-        <v>651</v>
+        <v>653</v>
       </c>
       <c r="J71" s="33" t="n">
-        <v>7</v>
+        <v>9.5</v>
       </c>
       <c r="K71" s="33" t="n">
-        <v>6308</v>
+        <v>8639</v>
       </c>
       <c r="L71" s="33" t="n">
-        <v>47.1</v>
+        <v>43.9</v>
       </c>
       <c r="M71" s="33" t="n">
-        <v>42613</v>
+        <v>39728</v>
       </c>
       <c r="N71" s="34" t="inlineStr">
         <is>
@@ -19547,34 +19601,34 @@
         <v>42205</v>
       </c>
       <c r="D72" s="33" t="n">
-        <v>60.2</v>
+        <v>38.4</v>
       </c>
       <c r="E72" s="33" t="n">
-        <v>25388</v>
+        <v>16198</v>
       </c>
       <c r="F72" s="33" t="n">
-        <v>27.5</v>
+        <v>43.4</v>
       </c>
       <c r="G72" s="33" t="n">
-        <v>11626</v>
+        <v>18303</v>
       </c>
       <c r="H72" s="33" t="n">
-        <v>4.5</v>
+        <v>14.1</v>
       </c>
       <c r="I72" s="33" t="n">
-        <v>1894</v>
+        <v>5946</v>
       </c>
       <c r="J72" s="33" t="n">
-        <v>7.8</v>
+        <v>4.2</v>
       </c>
       <c r="K72" s="33" t="n">
-        <v>3297</v>
+        <v>1758</v>
       </c>
       <c r="L72" s="33" t="n">
-        <v>39.8</v>
+        <v>61.6</v>
       </c>
       <c r="M72" s="33" t="n">
-        <v>16817</v>
+        <v>26007</v>
       </c>
       <c r="N72" s="34" t="inlineStr">
         <is>
@@ -19806,34 +19860,34 @@
         <v>21183</v>
       </c>
       <c r="D73" s="33" t="n">
-        <v>60.2</v>
+        <v>62.2</v>
       </c>
       <c r="E73" s="33" t="n">
-        <v>12742</v>
+        <v>13174</v>
       </c>
       <c r="F73" s="33" t="n">
-        <v>27.5</v>
+        <v>18.8</v>
       </c>
       <c r="G73" s="33" t="n">
-        <v>5835</v>
+        <v>3976</v>
       </c>
       <c r="H73" s="33" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="I73" s="33" t="n">
+        <v>3086</v>
+      </c>
+      <c r="J73" s="33" t="n">
         <v>4.5</v>
       </c>
-      <c r="I73" s="33" t="n">
-        <v>950</v>
-      </c>
-      <c r="J73" s="33" t="n">
-        <v>7.8</v>
-      </c>
       <c r="K73" s="33" t="n">
-        <v>1655</v>
+        <v>947</v>
       </c>
       <c r="L73" s="33" t="n">
-        <v>39.8</v>
+        <v>37.8</v>
       </c>
       <c r="M73" s="33" t="n">
-        <v>8440</v>
+        <v>8008</v>
       </c>
       <c r="N73" s="34" t="inlineStr">
         <is>
@@ -20083,34 +20137,34 @@
         <v>30208</v>
       </c>
       <c r="D74" s="33" t="n">
-        <v>60.2</v>
+        <v>52.2</v>
       </c>
       <c r="E74" s="33" t="n">
-        <v>18172</v>
+        <v>15772</v>
       </c>
       <c r="F74" s="33" t="n">
-        <v>27.5</v>
+        <v>38.8</v>
       </c>
       <c r="G74" s="33" t="n">
-        <v>8321</v>
+        <v>11732</v>
       </c>
       <c r="H74" s="33" t="n">
-        <v>4.5</v>
+        <v>0.3</v>
       </c>
       <c r="I74" s="33" t="n">
-        <v>1355</v>
+        <v>77</v>
       </c>
       <c r="J74" s="33" t="n">
-        <v>7.8</v>
+        <v>8.699999999999999</v>
       </c>
       <c r="K74" s="33" t="n">
-        <v>2360</v>
+        <v>2627</v>
       </c>
       <c r="L74" s="33" t="n">
-        <v>39.8</v>
+        <v>47.8</v>
       </c>
       <c r="M74" s="33" t="n">
-        <v>12037</v>
+        <v>14436</v>
       </c>
       <c r="N74" s="34" t="inlineStr">
         <is>
@@ -20342,38 +20396,38 @@
         <v>24296</v>
       </c>
       <c r="D75" s="33" t="n">
-        <v>60.2</v>
+        <v>94.5</v>
       </c>
       <c r="E75" s="33" t="n">
-        <v>14615</v>
+        <v>22955</v>
       </c>
       <c r="F75" s="33" t="n">
-        <v>27.5</v>
+        <v>4.8</v>
       </c>
       <c r="G75" s="33" t="n">
-        <v>6693</v>
+        <v>1163</v>
       </c>
       <c r="H75" s="33" t="n">
-        <v>4.5</v>
+        <v>0.4</v>
       </c>
       <c r="I75" s="33" t="n">
-        <v>1090</v>
+        <v>93</v>
       </c>
       <c r="J75" s="33" t="n">
-        <v>7.8</v>
+        <v>0.4</v>
       </c>
       <c r="K75" s="33" t="n">
-        <v>1898</v>
+        <v>85</v>
       </c>
       <c r="L75" s="33" t="n">
-        <v>39.8</v>
+        <v>5.5</v>
       </c>
       <c r="M75" s="33" t="n">
-        <v>9681</v>
+        <v>1341</v>
       </c>
       <c r="N75" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1-2</t>
         </is>
       </c>
       <c r="O75" s="35" t="n">
@@ -20601,34 +20655,34 @@
         <v>15675</v>
       </c>
       <c r="D76" s="33" t="n">
-        <v>60.2</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="E76" s="33" t="n">
-        <v>9429</v>
+        <v>12288</v>
       </c>
       <c r="F76" s="33" t="n">
-        <v>27.5</v>
+        <v>16.4</v>
       </c>
       <c r="G76" s="33" t="n">
-        <v>4318</v>
+        <v>2564</v>
       </c>
       <c r="H76" s="33" t="n">
-        <v>4.5</v>
+        <v>0</v>
       </c>
       <c r="I76" s="33" t="n">
-        <v>703</v>
+        <v>0</v>
       </c>
       <c r="J76" s="33" t="n">
-        <v>7.8</v>
+        <v>5.2</v>
       </c>
       <c r="K76" s="33" t="n">
-        <v>1225</v>
+        <v>823</v>
       </c>
       <c r="L76" s="33" t="n">
-        <v>39.8</v>
+        <v>21.6</v>
       </c>
       <c r="M76" s="33" t="n">
-        <v>6246</v>
+        <v>3386</v>
       </c>
       <c r="N76" s="34" t="inlineStr">
         <is>
@@ -20860,34 +20914,34 @@
         <v>22929</v>
       </c>
       <c r="D77" s="33" t="n">
-        <v>60.2</v>
+        <v>78</v>
       </c>
       <c r="E77" s="33" t="n">
-        <v>13793</v>
+        <v>17886</v>
       </c>
       <c r="F77" s="33" t="n">
-        <v>27.5</v>
+        <v>21.2</v>
       </c>
       <c r="G77" s="33" t="n">
-        <v>6316</v>
+        <v>4871</v>
       </c>
       <c r="H77" s="33" t="n">
-        <v>4.5</v>
+        <v>0.3</v>
       </c>
       <c r="I77" s="33" t="n">
-        <v>1029</v>
+        <v>67</v>
       </c>
       <c r="J77" s="33" t="n">
-        <v>7.8</v>
+        <v>0.5</v>
       </c>
       <c r="K77" s="33" t="n">
-        <v>1791</v>
+        <v>105</v>
       </c>
       <c r="L77" s="33" t="n">
-        <v>39.8</v>
+        <v>22</v>
       </c>
       <c r="M77" s="33" t="n">
-        <v>9136</v>
+        <v>5043</v>
       </c>
       <c r="N77" s="34" t="inlineStr">
         <is>
@@ -21116,42 +21170,40 @@
         </is>
       </c>
       <c r="C78" s="33" t="n">
-        <v>18250</v>
+        <v/>
       </c>
       <c r="D78" s="33" t="n">
-        <v>60.2</v>
+        <v/>
       </c>
       <c r="E78" s="33" t="n">
-        <v>10978</v>
+        <v/>
       </c>
       <c r="F78" s="33" t="n">
-        <v>27.5</v>
+        <v/>
       </c>
       <c r="G78" s="33" t="n">
-        <v>5027</v>
+        <v/>
       </c>
       <c r="H78" s="33" t="n">
-        <v>4.5</v>
+        <v/>
       </c>
       <c r="I78" s="33" t="n">
-        <v>819</v>
+        <v/>
       </c>
       <c r="J78" s="33" t="n">
-        <v>7.8</v>
+        <v/>
       </c>
       <c r="K78" s="33" t="n">
-        <v>1426</v>
+        <v/>
       </c>
       <c r="L78" s="33" t="n">
-        <v>39.8</v>
+        <v/>
       </c>
       <c r="M78" s="33" t="n">
-        <v>7272</v>
-      </c>
-      <c r="N78" s="34" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
+        <v/>
+      </c>
+      <c r="N78" s="34" t="n">
+        <v/>
       </c>
       <c r="O78" s="35" t="n">
         <v/>
@@ -21395,8 +21447,10 @@
       <c r="CB78" s="48" t="n">
         <v>0.4700319186665091</v>
       </c>
-      <c r="CC78" s="49" t="n">
-        <v>0.6402050147818953</v>
+      <c r="CC78" s="49" t="inlineStr">
+        <is>
+          <t>&lt;NA&gt;</t>
+        </is>
       </c>
     </row>
     <row r="79">
@@ -21414,34 +21468,34 @@
         <v>22986</v>
       </c>
       <c r="D79" s="33" t="n">
-        <v>60.2</v>
+        <v>42.8</v>
       </c>
       <c r="E79" s="33" t="n">
-        <v>13827</v>
+        <v>9840</v>
       </c>
       <c r="F79" s="33" t="n">
-        <v>27.5</v>
+        <v>55.6</v>
       </c>
       <c r="G79" s="33" t="n">
-        <v>6332</v>
+        <v>12777</v>
       </c>
       <c r="H79" s="33" t="n">
-        <v>4.5</v>
+        <v>1.6</v>
       </c>
       <c r="I79" s="33" t="n">
-        <v>1031</v>
+        <v>369</v>
       </c>
       <c r="J79" s="33" t="n">
-        <v>7.8</v>
+        <v>0</v>
       </c>
       <c r="K79" s="33" t="n">
-        <v>1796</v>
+        <v>0</v>
       </c>
       <c r="L79" s="33" t="n">
-        <v>39.8</v>
+        <v>57.2</v>
       </c>
       <c r="M79" s="33" t="n">
-        <v>9159</v>
+        <v>13147</v>
       </c>
       <c r="N79" s="34" t="inlineStr">
         <is>
@@ -21673,38 +21727,38 @@
         <v>31031</v>
       </c>
       <c r="D80" s="33" t="n">
-        <v>60.2</v>
+        <v>33.1</v>
       </c>
       <c r="E80" s="33" t="n">
-        <v>18666</v>
+        <v>10285</v>
       </c>
       <c r="F80" s="33" t="n">
-        <v>27.5</v>
+        <v>26.3</v>
       </c>
       <c r="G80" s="33" t="n">
-        <v>8548</v>
+        <v>8175</v>
       </c>
       <c r="H80" s="33" t="n">
-        <v>4.5</v>
+        <v>1.2</v>
       </c>
       <c r="I80" s="33" t="n">
-        <v>1392</v>
+        <v>359</v>
       </c>
       <c r="J80" s="33" t="n">
-        <v>7.8</v>
+        <v>39.4</v>
       </c>
       <c r="K80" s="33" t="n">
-        <v>2424</v>
+        <v>12212</v>
       </c>
       <c r="L80" s="33" t="n">
-        <v>39.8</v>
+        <v>66.90000000000001</v>
       </c>
       <c r="M80" s="33" t="n">
-        <v>12365</v>
+        <v>20746</v>
       </c>
       <c r="N80" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O80" s="35" t="n">
@@ -21932,38 +21986,38 @@
         <v>44663</v>
       </c>
       <c r="D81" s="33" t="n">
-        <v>60.2</v>
+        <v>41.4</v>
       </c>
       <c r="E81" s="33" t="n">
-        <v>26867</v>
+        <v>18491</v>
       </c>
       <c r="F81" s="33" t="n">
-        <v>27.5</v>
+        <v>21.4</v>
       </c>
       <c r="G81" s="33" t="n">
-        <v>12303</v>
+        <v>9554</v>
       </c>
       <c r="H81" s="33" t="n">
-        <v>4.5</v>
+        <v>8</v>
       </c>
       <c r="I81" s="33" t="n">
-        <v>2004</v>
+        <v>3587</v>
       </c>
       <c r="J81" s="33" t="n">
-        <v>7.8</v>
+        <v>29.2</v>
       </c>
       <c r="K81" s="33" t="n">
-        <v>3490</v>
+        <v>13031</v>
       </c>
       <c r="L81" s="33" t="n">
-        <v>39.8</v>
+        <v>58.6</v>
       </c>
       <c r="M81" s="33" t="n">
-        <v>17797</v>
+        <v>26172</v>
       </c>
       <c r="N81" s="34" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="O81" s="35" t="n">

</xml_diff>